<commit_message>
update - 11/06/2026 15:40
</commit_message>
<xml_diff>
--- a/ADL_Timesheet_Template.xlsx
+++ b/ADL_Timesheet_Template.xlsx
@@ -10,9 +10,10 @@
   <sheets>
     <sheet name="Instructions" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Timesheet" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="_Lists" sheetId="3" state="hidden" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Titles" vbProcedure="false">Timesheet!$9:$9</definedName>
+    <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Titles" vbProcedure="false">Timesheet!$10:$10</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="76">
   <si>
     <t xml:space="preserve">AXIOM DL — TIMESHEET INSTRUCTIONS</t>
   </si>
@@ -35,29 +36,22 @@
     <t xml:space="preserve">  1 — GETTING STARTED</t>
   </si>
   <si>
-    <t xml:space="preserve">Template file</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Use this template every time. Do not add, remove, or rename columns.</t>
-  </si>
-  <si>
     <t xml:space="preserve">File naming</t>
   </si>
   <si>
-    <t xml:space="preserve">Save as: YYYY-WXX_FirstnameLastname.xlsx
-Example: 2026-W24_GreigFensome.xlsx</t>
+    <t xml:space="preserve">Save as: YYYY-WXX_FirstnameLastname.xlsx  e.g. 2026-W24_GreigFensome.xlsx</t>
   </si>
   <si>
     <t xml:space="preserve">One file per week</t>
   </si>
   <si>
-    <t xml:space="preserve">Submit one file covering Mon–Fri for the week. Do not combine multiple weeks.</t>
+    <t xml:space="preserve">Submit one file covering Mon–Fri. Do not combine multiple weeks.</t>
   </si>
   <si>
     <t xml:space="preserve">Where to upload</t>
   </si>
   <si>
-    <t xml:space="preserve">Dropbox: /Timesheets/Inbox/  — do not upload to any other folder.</t>
+    <t xml:space="preserve">Dropbox: /Timesheets/Inbox/ — do not upload to any other folder.</t>
   </si>
   <si>
     <t xml:space="preserve">Submission deadline</t>
@@ -72,26 +66,37 @@
     <t xml:space="preserve">Name</t>
   </si>
   <si>
-    <t xml:space="preserve">Enter your full name in the Name field at the top. Must match Notion exactly.</t>
+    <t xml:space="preserve">Enter your full name exactly as it appears in Notion.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Week Commencing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enter the Monday date for the week. Week number and range auto-fill.</t>
   </si>
   <si>
     <t xml:space="preserve">Date</t>
   </si>
   <si>
-    <t xml:space="preserve">Select from the date picker. Format: DD/MM/YYYY. All dates must fall within the same week.</t>
+    <t xml:space="preserve">Click the cell and use the date selector. All dates must fall within the same week.</t>
   </si>
   <si>
     <t xml:space="preserve">Day</t>
   </si>
   <si>
-    <t xml:space="preserve">Choose from the dropdown (Mon–Sun). Auto-fills if you enter the date first.</t>
+    <t xml:space="preserve">Auto-populated from the Date — do not edit.</t>
   </si>
   <si>
     <t xml:space="preserve">Project</t>
   </si>
   <si>
-    <t xml:space="preserve">Enter the full project reference: YY-NNN or YY-NNN Project Name
-Example: 24-367 EIT Observation Hall</t>
+    <t xml:space="preserve">Full project reference: YY-NNN or YY-NNN Project Name  e.g. 24-367 EIT Observation Hall</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Item No.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The drawing or deliverable item number if applicable (e.g. SK-001, DR-045). Leave blank if not relevant.</t>
   </si>
   <si>
     <t xml:space="preserve">Category</t>
@@ -103,7 +108,7 @@
     <t xml:space="preserve">Description</t>
   </si>
   <si>
-    <t xml:space="preserve">Brief description of the work done. Be specific — 'detailed design of entrance lobby' not 'design work'.</t>
+    <t xml:space="preserve">Brief description of work done. Be specific — 'curtain wall detail design' not 'design work'.</t>
   </si>
   <si>
     <t xml:space="preserve">Hours</t>
@@ -112,55 +117,73 @@
     <t xml:space="preserve">Decimal format only: 0.5, 1.0, 7.5. Not HH:MM. Max 24 per row.</t>
   </si>
   <si>
-    <t xml:space="preserve">Blank rows</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Leave unused rows blank. Do not delete them.</t>
-  </si>
-  <si>
     <t xml:space="preserve">  3 — CATEGORY DEFINITIONS</t>
   </si>
   <si>
-    <t xml:space="preserve">Design</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Concept design, architectural design, detailed design, design development.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Drafting</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAD work, Revit modelling, technical drawing, detailing, AutoCAD drafting.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Coordination</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Technical coordination, clash detection, co-ordination with other disciplines.</t>
+    <t xml:space="preserve">Coordination &amp; Research</t>
+  </si>
+  <si>
+    <t xml:space="preserve">General project coordination, research, information gathering, RFIs, technical queries.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Drawing &amp; Modelling - Production</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Active production of new drawings or models — first-time creation of a deliverable.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Drawing &amp; Modelling - Revision</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Revising or updating an existing drawing or model following comments or design changes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Drawing &amp; Modelling - First Issue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Final checking, packaging, and issuing a drawing or model for the first time.</t>
   </si>
   <si>
     <t xml:space="preserve">Meetings</t>
   </si>
   <si>
-    <t xml:space="preserve">Client meetings, design team meetings, calls, site visits involving meetings.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Admin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Project management, emails, programme tracking, resource planning.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Site</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Site surveys, site inspections, on-site visits not covered by Meetings.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Other</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Anything not covered above. Add a clear description.</t>
+    <t xml:space="preserve">All meetings — client, design team, internal, calls, video conferences.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DM Development</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Design management activities focused on developing the project delivery strategy.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DM Coordination</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Design management coordination — managing information flow between disciplines.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DM Project Admin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Project administration tasks: programmes, trackers, reports, correspondence.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DM Meetings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Design management specific meetings — not covered under general Meetings.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Document Control</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Document control activities: transmittals, registers, file management.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Travel Time</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Time spent travelling to/from site, client offices, or other project locations.</t>
   </si>
   <si>
     <t xml:space="preserve">  4 — PROJECT REFERENCES</t>
@@ -175,55 +198,34 @@
     <t xml:space="preserve">Project name</t>
   </si>
   <si>
-    <t xml:space="preserve">You may append the project name after the ref: 24-367 EIT Observation Hall.</t>
+    <t xml:space="preserve">You may append the name after the ref: 24-367 EIT Observation Hall.</t>
   </si>
   <si>
     <t xml:space="preserve">No ref available</t>
   </si>
   <si>
-    <t xml:space="preserve">Use 'INTERNAL' for internal/overhead work with no project number.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Unknown ref</t>
-  </si>
-  <si>
-    <t xml:space="preserve">If you are unsure of the project number, mark the row and contact your PM.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  5 — COMMON MISTAKES TO AVOID</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Wrong column format</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Do not enter time as HH:MM (e.g. 7:30). Use decimal hours (7.5).</t>
+    <t xml:space="preserve">Use INTERNAL for overhead/non-project work.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  5 — COMMON MISTAKES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hours as HH:MM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enter 7.5 not 07:30. Incorrect format will be flagged on import.</t>
   </si>
   <si>
     <t xml:space="preserve">Missing project ref</t>
   </si>
   <si>
-    <t xml:space="preserve">Rows without a valid project ref will be flagged on import and need manual review.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Renaming the file wrong</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Wrong filename = import failure. Check: YYYY-WXX_FirstnameLastname.xlsx.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Wrong Dropbox folder</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Only /Timesheets/Inbox/ is scanned. Files in any other folder will not be picked up.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  6 — QUESTIONS &amp; SUPPORT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Contact</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Speak to your project manager or contact the studio admin.</t>
+    <t xml:space="preserve">Rows without a project ref are flagged and require manual review.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Editing Day column</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Day is a formula — do not type into it. It auto-fills from Date.</t>
   </si>
   <si>
     <t xml:space="preserve">AXIOM DL — TIMESHEET</t>
@@ -232,13 +234,13 @@
     <t xml:space="preserve">Name:</t>
   </si>
   <si>
-    <t xml:space="preserve">Week:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">e.g. 2026-W24  (Mon 08/06 – Fri 12/06)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  ⚠  Fill in amber cells. Use dropdown lists for Day and Category. Hours must be in decimal format (e.g. 7.5). Upload to Dropbox: /Timesheets/Inbox/</t>
+    <t xml:space="preserve">Wk Commencing:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ISO Week:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  ⚠  Amber cells = user input. Blue cells = auto-calculated — do not edit. Upload to: Dropbox /Timesheets/Inbox/</t>
   </si>
   <si>
     <t xml:space="preserve">#</t>
@@ -250,7 +252,7 @@
     <t xml:space="preserve">TOTAL</t>
   </si>
   <si>
-    <t xml:space="preserve">  File naming: YYYY-WXX_FirstnameLastname.xlsx  |  Upload to: Dropbox /Timesheets/Inbox/  |  Deadline: Monday 09:00 for previous week</t>
+    <t xml:space="preserve">  File naming: YYYY-WXX_FirstnameLastname.xlsx  |  Upload to: Dropbox /Timesheets/Inbox/  |  Deadline: Monday 09:00</t>
   </si>
 </sst>
 </file>
@@ -262,7 +264,7 @@
     <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="166" formatCode="0.0"/>
   </numFmts>
-  <fonts count="18">
+  <fonts count="19">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -333,9 +335,16 @@
       <charset val="1"/>
     </font>
     <font>
-      <i val="true"/>
-      <sz val="9"/>
-      <color rgb="FF6B7280"/>
+      <sz val="10"/>
+      <color rgb="FF1A1A2E"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="10"/>
+      <color rgb="FF1B3A6B"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -365,14 +374,13 @@
     </font>
     <font>
       <sz val="10"/>
+      <color rgb="FF1B3A6B"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
       <sz val="10"/>
-      <color rgb="FF1B3A6B"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -394,7 +402,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -422,7 +430,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF2F6FC"/>
-        <bgColor rgb="FFF5F5F5"/>
+        <bgColor rgb="FFEFF6FF"/>
       </patternFill>
     </fill>
     <fill>
@@ -439,6 +447,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFEFF6FF"/>
+        <bgColor rgb="FFF2F6FC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFFF3CD"/>
         <bgColor rgb="FFFFF8E7"/>
       </patternFill>
@@ -446,11 +460,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFD6E4F7"/>
-        <bgColor rgb="FFF2F6FC"/>
+        <bgColor rgb="FFEFF6FF"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="8">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -491,6 +505,21 @@
         <color rgb="FF2E5FA3"/>
       </left>
       <right/>
+      <top style="medium">
+        <color rgb="FF2E5FA3"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF2E5FA3"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="medium">
+        <color rgb="FF2E5FA3"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF2E5FA3"/>
+      </right>
       <top style="medium">
         <color rgb="FF2E5FA3"/>
       </top>
@@ -568,7 +597,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="32">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -617,35 +646,47 @@
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="7" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="10" fillId="7" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="8" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="10" fillId="7" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="2" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="8" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="9" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="2" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="4" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="7" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="15" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -653,15 +694,15 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="5" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="5" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -669,19 +710,19 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="9" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="10" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="9" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="10" borderId="7" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="16" fillId="9" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="17" fillId="10" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="18" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -715,7 +756,7 @@
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FFFFF3CD"/>
-      <rgbColor rgb="FFF2F6FC"/>
+      <rgbColor rgb="FFEFF6FF"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
       <rgbColor rgb="FF2E5FA3"/>
@@ -729,8 +770,8 @@
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FF00CCFF"/>
+      <rgbColor rgb="FFF2F6FC"/>
       <rgbColor rgb="FFF5F5F5"/>
-      <rgbColor rgb="FFCCFFCC"/>
       <rgbColor rgb="FFFFF8E7"/>
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
@@ -938,23 +979,22 @@
     <tabColor rgb="FF2E5FA3"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D47"/>
+  <dimension ref="A2:D45"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="60"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="3"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
     </row>
-    <row r="3" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="1"/>
       <c r="B3" s="2" t="s">
         <v>0</v>
@@ -962,7 +1002,7 @@
       <c r="C3" s="2"/>
       <c r="D3" s="1"/>
     </row>
-    <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
@@ -976,290 +1016,289 @@
       <c r="C5" s="4"/>
       <c r="D5" s="3"/>
     </row>
-    <row r="7" customFormat="false" ht="7.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="8" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B8" s="5" t="s">
+    <row r="7" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B7" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="C8" s="5"/>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B9" s="6" t="s">
+      <c r="C7" s="5"/>
+    </row>
+    <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B8" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C8" s="7" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B10" s="8" t="s">
+    <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B9" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="C10" s="9" t="s">
+      <c r="C9" s="9" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B11" s="6" t="s">
+    <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B10" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="C10" s="7" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B12" s="8" t="s">
+    <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B11" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="C12" s="9" t="s">
+      <c r="C11" s="9" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B13" s="6" t="s">
+    <row r="12" customFormat="false" ht="6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="13" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B13" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C13" s="7" t="s">
+      <c r="C13" s="5"/>
+    </row>
+    <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B14" s="6" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="14" customFormat="false" ht="7.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="15" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B15" s="5" t="s">
+      <c r="C14" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="C15" s="5"/>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B15" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C15" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="6" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B17" s="8" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B18" s="6" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B19" s="8" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C19" s="9" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B20" s="6" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B21" s="8" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B22" s="6" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B23" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="C23" s="9" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="7.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="25" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B25" s="5" t="s">
+    <row r="23" customFormat="false" ht="6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B24" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="C25" s="5"/>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C24" s="5"/>
+    </row>
+    <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B25" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="C25" s="7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B26" s="6" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B27" s="8" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B28" s="6" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B29" s="8" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C29" s="9" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B30" s="6" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B31" s="8" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C31" s="9" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B32" s="6" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C32" s="7" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="7.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="34" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B34" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="C34" s="5"/>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B35" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="C35" s="7" t="s">
+    </row>
+    <row r="33" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B33" s="8" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B36" s="8" t="s">
+      <c r="C33" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="C36" s="9" t="s">
+    </row>
+    <row r="34" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B34" s="6" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B37" s="6" t="s">
+      <c r="C34" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="C37" s="7" t="s">
+    </row>
+    <row r="35" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B35" s="8" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B38" s="8" t="s">
+      <c r="C35" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="C38" s="9" t="s">
+    </row>
+    <row r="36" customFormat="false" ht="6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="37" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B37" s="5" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="39" customFormat="false" ht="7.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="40" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B40" s="5" t="s">
+      <c r="C37" s="5"/>
+    </row>
+    <row r="38" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B38" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="C40" s="5"/>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B41" s="6" t="s">
+      <c r="C38" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="C41" s="7" t="s">
+    </row>
+    <row r="39" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B39" s="8" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B42" s="8" t="s">
+      <c r="C39" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="C42" s="9" t="s">
+    </row>
+    <row r="40" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B40" s="6" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C40" s="7" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="42" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B42" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C42" s="5"/>
+    </row>
+    <row r="43" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B43" s="6" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C43" s="7" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B44" s="8" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C44" s="9" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="45" customFormat="false" ht="7.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="46" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B46" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="C46" s="5"/>
-    </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B47" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="C47" s="7" t="s">
+    </row>
+    <row r="45" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B45" s="6" t="s">
         <v>65</v>
       </c>
+      <c r="C45" s="7" t="s">
+        <v>66</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="7">
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="B34:C34"/>
-    <mergeCell ref="B40:C40"/>
-    <mergeCell ref="B46:C46"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="B42:C42"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1277,17 +1316,17 @@
     <tabColor rgb="FF1B3A6B"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:H42"/>
+  <dimension ref="A1:H43"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="9"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="7.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1302,7 +1341,7 @@
     </row>
     <row r="2" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B2" s="10"/>
       <c r="C2" s="10"/>
@@ -1310,7 +1349,7 @@
       <c r="E2" s="10"/>
       <c r="F2" s="10"/>
       <c r="G2" s="10"/>
-      <c r="H2" s="1"/>
+      <c r="H2" s="10"/>
     </row>
     <row r="3" customFormat="false" ht="7.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3"/>
@@ -1325,433 +1364,567 @@
     <row r="4" customFormat="false" ht="4.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="5" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B5" s="12"/>
       <c r="C5" s="12"/>
       <c r="D5" s="12"/>
-      <c r="E5" s="11" t="s">
-        <v>68</v>
-      </c>
-      <c r="F5" s="13" t="s">
+    </row>
+    <row r="6" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="G5" s="13"/>
-    </row>
-    <row r="6" customFormat="false" ht="4.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="14" t="s">
+      <c r="B6" s="13"/>
+      <c r="E6" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="B7" s="14"/>
-      <c r="C7" s="14"/>
-      <c r="D7" s="14"/>
-      <c r="E7" s="14"/>
-      <c r="F7" s="14"/>
-      <c r="G7" s="14"/>
-    </row>
-    <row r="8" customFormat="false" ht="4.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="9" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="15" t="s">
+      <c r="F6" s="14" t="str">
+        <f aca="false">IF(B6="","",YEAR(B6+3-WEEKDAY(B6,2))&amp;"-W"&amp;TEXT(isoweeknum(B6),"00")&amp;"  ("&amp;TEXT(B6,"DD/MM")&amp;" – "&amp;TEXT(B6+4,"DD/MM")&amp;")")</f>
+        <v/>
+      </c>
+      <c r="G6" s="14"/>
+      <c r="H6" s="14"/>
+    </row>
+    <row r="7" customFormat="false" ht="4.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="15" t="s">
         <v>71</v>
       </c>
-      <c r="B9" s="15" t="s">
+      <c r="B8" s="15"/>
+      <c r="C8" s="15"/>
+      <c r="D8" s="15"/>
+      <c r="E8" s="15"/>
+      <c r="F8" s="15"/>
+      <c r="G8" s="15"/>
+      <c r="H8" s="15"/>
+    </row>
+    <row r="9" customFormat="false" ht="4.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="10" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="16" t="s">
+        <v>72</v>
+      </c>
+      <c r="B10" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="C9" s="15" t="s">
+      <c r="C10" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="D9" s="15" t="s">
-        <v>72</v>
-      </c>
-      <c r="E9" s="15" t="s">
+      <c r="D10" s="16" t="s">
+        <v>73</v>
+      </c>
+      <c r="E10" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="F9" s="15" t="s">
+      <c r="F10" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="G9" s="15" t="s">
+      <c r="G10" s="16" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="10" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="16" t="n">
+      <c r="H10" s="16" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="B10" s="17"/>
-      <c r="C10" s="18"/>
-      <c r="D10" s="19"/>
-      <c r="E10" s="18"/>
-      <c r="F10" s="19"/>
-      <c r="G10" s="20"/>
-    </row>
-    <row r="11" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="16" t="n">
+      <c r="B11" s="18"/>
+      <c r="C11" s="19" t="str">
+        <f aca="false">IF(B11="","",TEXT(B11,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="D11" s="20"/>
+      <c r="E11" s="21"/>
+      <c r="F11" s="22"/>
+      <c r="G11" s="20"/>
+      <c r="H11" s="23"/>
+    </row>
+    <row r="12" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="B11" s="21"/>
-      <c r="C11" s="22"/>
-      <c r="D11" s="23"/>
-      <c r="E11" s="22"/>
-      <c r="F11" s="23"/>
-      <c r="G11" s="24"/>
-    </row>
-    <row r="12" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="16" t="n">
+      <c r="B12" s="18"/>
+      <c r="C12" s="19" t="str">
+        <f aca="false">IF(B12="","",TEXT(B12,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="D12" s="24"/>
+      <c r="E12" s="25"/>
+      <c r="F12" s="26"/>
+      <c r="G12" s="24"/>
+      <c r="H12" s="27"/>
+    </row>
+    <row r="13" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="17" t="n">
         <v>3</v>
       </c>
-      <c r="B12" s="17"/>
-      <c r="C12" s="18"/>
-      <c r="D12" s="19"/>
-      <c r="E12" s="18"/>
-      <c r="F12" s="19"/>
-      <c r="G12" s="20"/>
-    </row>
-    <row r="13" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="16" t="n">
+      <c r="B13" s="18"/>
+      <c r="C13" s="19" t="str">
+        <f aca="false">IF(B13="","",TEXT(B13,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="D13" s="20"/>
+      <c r="E13" s="21"/>
+      <c r="F13" s="22"/>
+      <c r="G13" s="20"/>
+      <c r="H13" s="23"/>
+    </row>
+    <row r="14" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="17" t="n">
         <v>4</v>
       </c>
-      <c r="B13" s="21"/>
-      <c r="C13" s="22"/>
-      <c r="D13" s="23"/>
-      <c r="E13" s="22"/>
-      <c r="F13" s="23"/>
-      <c r="G13" s="24"/>
-    </row>
-    <row r="14" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="16" t="n">
+      <c r="B14" s="18"/>
+      <c r="C14" s="19" t="str">
+        <f aca="false">IF(B14="","",TEXT(B14,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="D14" s="24"/>
+      <c r="E14" s="25"/>
+      <c r="F14" s="26"/>
+      <c r="G14" s="24"/>
+      <c r="H14" s="27"/>
+    </row>
+    <row r="15" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="17" t="n">
         <v>5</v>
       </c>
-      <c r="B14" s="17"/>
-      <c r="C14" s="18"/>
-      <c r="D14" s="19"/>
-      <c r="E14" s="18"/>
-      <c r="F14" s="19"/>
-      <c r="G14" s="20"/>
-    </row>
-    <row r="15" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="16" t="n">
+      <c r="B15" s="18"/>
+      <c r="C15" s="19" t="str">
+        <f aca="false">IF(B15="","",TEXT(B15,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="D15" s="20"/>
+      <c r="E15" s="21"/>
+      <c r="F15" s="22"/>
+      <c r="G15" s="20"/>
+      <c r="H15" s="23"/>
+    </row>
+    <row r="16" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="17" t="n">
         <v>6</v>
       </c>
-      <c r="B15" s="21"/>
-      <c r="C15" s="22"/>
-      <c r="D15" s="23"/>
-      <c r="E15" s="22"/>
-      <c r="F15" s="23"/>
-      <c r="G15" s="24"/>
-    </row>
-    <row r="16" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="16" t="n">
+      <c r="B16" s="18"/>
+      <c r="C16" s="19" t="str">
+        <f aca="false">IF(B16="","",TEXT(B16,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="D16" s="24"/>
+      <c r="E16" s="25"/>
+      <c r="F16" s="26"/>
+      <c r="G16" s="24"/>
+      <c r="H16" s="27"/>
+    </row>
+    <row r="17" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="17" t="n">
         <v>7</v>
       </c>
-      <c r="B16" s="17"/>
-      <c r="C16" s="18"/>
-      <c r="D16" s="19"/>
-      <c r="E16" s="18"/>
-      <c r="F16" s="19"/>
-      <c r="G16" s="20"/>
-    </row>
-    <row r="17" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="16" t="n">
+      <c r="B17" s="18"/>
+      <c r="C17" s="19" t="str">
+        <f aca="false">IF(B17="","",TEXT(B17,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="D17" s="20"/>
+      <c r="E17" s="21"/>
+      <c r="F17" s="22"/>
+      <c r="G17" s="20"/>
+      <c r="H17" s="23"/>
+    </row>
+    <row r="18" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="17" t="n">
         <v>8</v>
       </c>
-      <c r="B17" s="21"/>
-      <c r="C17" s="22"/>
-      <c r="D17" s="23"/>
-      <c r="E17" s="22"/>
-      <c r="F17" s="23"/>
-      <c r="G17" s="24"/>
-    </row>
-    <row r="18" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="16" t="n">
+      <c r="B18" s="18"/>
+      <c r="C18" s="19" t="str">
+        <f aca="false">IF(B18="","",TEXT(B18,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="D18" s="24"/>
+      <c r="E18" s="25"/>
+      <c r="F18" s="26"/>
+      <c r="G18" s="24"/>
+      <c r="H18" s="27"/>
+    </row>
+    <row r="19" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="17" t="n">
         <v>9</v>
       </c>
-      <c r="B18" s="17"/>
-      <c r="C18" s="18"/>
-      <c r="D18" s="19"/>
-      <c r="E18" s="18"/>
-      <c r="F18" s="19"/>
-      <c r="G18" s="20"/>
-    </row>
-    <row r="19" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="16" t="n">
+      <c r="B19" s="18"/>
+      <c r="C19" s="19" t="str">
+        <f aca="false">IF(B19="","",TEXT(B19,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="D19" s="20"/>
+      <c r="E19" s="21"/>
+      <c r="F19" s="22"/>
+      <c r="G19" s="20"/>
+      <c r="H19" s="23"/>
+    </row>
+    <row r="20" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="17" t="n">
         <v>10</v>
       </c>
-      <c r="B19" s="21"/>
-      <c r="C19" s="22"/>
-      <c r="D19" s="23"/>
-      <c r="E19" s="22"/>
-      <c r="F19" s="23"/>
-      <c r="G19" s="24"/>
-    </row>
-    <row r="20" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="16" t="n">
+      <c r="B20" s="18"/>
+      <c r="C20" s="19" t="str">
+        <f aca="false">IF(B20="","",TEXT(B20,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="D20" s="24"/>
+      <c r="E20" s="25"/>
+      <c r="F20" s="26"/>
+      <c r="G20" s="24"/>
+      <c r="H20" s="27"/>
+    </row>
+    <row r="21" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="17" t="n">
         <v>11</v>
       </c>
-      <c r="B20" s="17"/>
-      <c r="C20" s="18"/>
-      <c r="D20" s="19"/>
-      <c r="E20" s="18"/>
-      <c r="F20" s="19"/>
-      <c r="G20" s="20"/>
-    </row>
-    <row r="21" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="16" t="n">
+      <c r="B21" s="18"/>
+      <c r="C21" s="19" t="str">
+        <f aca="false">IF(B21="","",TEXT(B21,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="D21" s="20"/>
+      <c r="E21" s="21"/>
+      <c r="F21" s="22"/>
+      <c r="G21" s="20"/>
+      <c r="H21" s="23"/>
+    </row>
+    <row r="22" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="17" t="n">
         <v>12</v>
       </c>
-      <c r="B21" s="21"/>
-      <c r="C21" s="22"/>
-      <c r="D21" s="23"/>
-      <c r="E21" s="22"/>
-      <c r="F21" s="23"/>
-      <c r="G21" s="24"/>
-    </row>
-    <row r="22" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="16" t="n">
+      <c r="B22" s="18"/>
+      <c r="C22" s="19" t="str">
+        <f aca="false">IF(B22="","",TEXT(B22,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="D22" s="24"/>
+      <c r="E22" s="25"/>
+      <c r="F22" s="26"/>
+      <c r="G22" s="24"/>
+      <c r="H22" s="27"/>
+    </row>
+    <row r="23" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="17" t="n">
         <v>13</v>
       </c>
-      <c r="B22" s="17"/>
-      <c r="C22" s="18"/>
-      <c r="D22" s="19"/>
-      <c r="E22" s="18"/>
-      <c r="F22" s="19"/>
-      <c r="G22" s="20"/>
-    </row>
-    <row r="23" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="16" t="n">
+      <c r="B23" s="18"/>
+      <c r="C23" s="19" t="str">
+        <f aca="false">IF(B23="","",TEXT(B23,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="D23" s="20"/>
+      <c r="E23" s="21"/>
+      <c r="F23" s="22"/>
+      <c r="G23" s="20"/>
+      <c r="H23" s="23"/>
+    </row>
+    <row r="24" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="17" t="n">
         <v>14</v>
       </c>
-      <c r="B23" s="21"/>
-      <c r="C23" s="22"/>
-      <c r="D23" s="23"/>
-      <c r="E23" s="22"/>
-      <c r="F23" s="23"/>
-      <c r="G23" s="24"/>
-    </row>
-    <row r="24" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="16" t="n">
+      <c r="B24" s="18"/>
+      <c r="C24" s="19" t="str">
+        <f aca="false">IF(B24="","",TEXT(B24,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="D24" s="24"/>
+      <c r="E24" s="25"/>
+      <c r="F24" s="26"/>
+      <c r="G24" s="24"/>
+      <c r="H24" s="27"/>
+    </row>
+    <row r="25" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="17" t="n">
         <v>15</v>
       </c>
-      <c r="B24" s="17"/>
-      <c r="C24" s="18"/>
-      <c r="D24" s="19"/>
-      <c r="E24" s="18"/>
-      <c r="F24" s="19"/>
-      <c r="G24" s="20"/>
-    </row>
-    <row r="25" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="16" t="n">
+      <c r="B25" s="18"/>
+      <c r="C25" s="19" t="str">
+        <f aca="false">IF(B25="","",TEXT(B25,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="D25" s="20"/>
+      <c r="E25" s="21"/>
+      <c r="F25" s="22"/>
+      <c r="G25" s="20"/>
+      <c r="H25" s="23"/>
+    </row>
+    <row r="26" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="17" t="n">
         <v>16</v>
       </c>
-      <c r="B25" s="21"/>
-      <c r="C25" s="22"/>
-      <c r="D25" s="23"/>
-      <c r="E25" s="22"/>
-      <c r="F25" s="23"/>
-      <c r="G25" s="24"/>
-    </row>
-    <row r="26" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="16" t="n">
+      <c r="B26" s="18"/>
+      <c r="C26" s="19" t="str">
+        <f aca="false">IF(B26="","",TEXT(B26,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="D26" s="24"/>
+      <c r="E26" s="25"/>
+      <c r="F26" s="26"/>
+      <c r="G26" s="24"/>
+      <c r="H26" s="27"/>
+    </row>
+    <row r="27" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="17" t="n">
         <v>17</v>
       </c>
-      <c r="B26" s="17"/>
-      <c r="C26" s="18"/>
-      <c r="D26" s="19"/>
-      <c r="E26" s="18"/>
-      <c r="F26" s="19"/>
-      <c r="G26" s="20"/>
-    </row>
-    <row r="27" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="16" t="n">
+      <c r="B27" s="18"/>
+      <c r="C27" s="19" t="str">
+        <f aca="false">IF(B27="","",TEXT(B27,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="D27" s="20"/>
+      <c r="E27" s="21"/>
+      <c r="F27" s="22"/>
+      <c r="G27" s="20"/>
+      <c r="H27" s="23"/>
+    </row>
+    <row r="28" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="17" t="n">
         <v>18</v>
       </c>
-      <c r="B27" s="21"/>
-      <c r="C27" s="22"/>
-      <c r="D27" s="23"/>
-      <c r="E27" s="22"/>
-      <c r="F27" s="23"/>
-      <c r="G27" s="24"/>
-    </row>
-    <row r="28" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="16" t="n">
+      <c r="B28" s="18"/>
+      <c r="C28" s="19" t="str">
+        <f aca="false">IF(B28="","",TEXT(B28,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="D28" s="24"/>
+      <c r="E28" s="25"/>
+      <c r="F28" s="26"/>
+      <c r="G28" s="24"/>
+      <c r="H28" s="27"/>
+    </row>
+    <row r="29" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="17" t="n">
         <v>19</v>
       </c>
-      <c r="B28" s="17"/>
-      <c r="C28" s="18"/>
-      <c r="D28" s="19"/>
-      <c r="E28" s="18"/>
-      <c r="F28" s="19"/>
-      <c r="G28" s="20"/>
-    </row>
-    <row r="29" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="16" t="n">
+      <c r="B29" s="18"/>
+      <c r="C29" s="19" t="str">
+        <f aca="false">IF(B29="","",TEXT(B29,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="D29" s="20"/>
+      <c r="E29" s="21"/>
+      <c r="F29" s="22"/>
+      <c r="G29" s="20"/>
+      <c r="H29" s="23"/>
+    </row>
+    <row r="30" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="17" t="n">
         <v>20</v>
       </c>
-      <c r="B29" s="21"/>
-      <c r="C29" s="22"/>
-      <c r="D29" s="23"/>
-      <c r="E29" s="22"/>
-      <c r="F29" s="23"/>
-      <c r="G29" s="24"/>
-    </row>
-    <row r="30" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="16" t="n">
+      <c r="B30" s="18"/>
+      <c r="C30" s="19" t="str">
+        <f aca="false">IF(B30="","",TEXT(B30,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="D30" s="24"/>
+      <c r="E30" s="25"/>
+      <c r="F30" s="26"/>
+      <c r="G30" s="24"/>
+      <c r="H30" s="27"/>
+    </row>
+    <row r="31" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="17" t="n">
         <v>21</v>
       </c>
-      <c r="B30" s="17"/>
-      <c r="C30" s="18"/>
-      <c r="D30" s="19"/>
-      <c r="E30" s="18"/>
-      <c r="F30" s="19"/>
-      <c r="G30" s="20"/>
-    </row>
-    <row r="31" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="16" t="n">
+      <c r="B31" s="18"/>
+      <c r="C31" s="19" t="str">
+        <f aca="false">IF(B31="","",TEXT(B31,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="D31" s="20"/>
+      <c r="E31" s="21"/>
+      <c r="F31" s="22"/>
+      <c r="G31" s="20"/>
+      <c r="H31" s="23"/>
+    </row>
+    <row r="32" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="17" t="n">
         <v>22</v>
       </c>
-      <c r="B31" s="21"/>
-      <c r="C31" s="22"/>
-      <c r="D31" s="23"/>
-      <c r="E31" s="22"/>
-      <c r="F31" s="23"/>
-      <c r="G31" s="24"/>
-    </row>
-    <row r="32" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="16" t="n">
+      <c r="B32" s="18"/>
+      <c r="C32" s="19" t="str">
+        <f aca="false">IF(B32="","",TEXT(B32,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="D32" s="24"/>
+      <c r="E32" s="25"/>
+      <c r="F32" s="26"/>
+      <c r="G32" s="24"/>
+      <c r="H32" s="27"/>
+    </row>
+    <row r="33" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="17" t="n">
         <v>23</v>
       </c>
-      <c r="B32" s="17"/>
-      <c r="C32" s="18"/>
-      <c r="D32" s="19"/>
-      <c r="E32" s="18"/>
-      <c r="F32" s="19"/>
-      <c r="G32" s="20"/>
-    </row>
-    <row r="33" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="16" t="n">
+      <c r="B33" s="18"/>
+      <c r="C33" s="19" t="str">
+        <f aca="false">IF(B33="","",TEXT(B33,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="D33" s="20"/>
+      <c r="E33" s="21"/>
+      <c r="F33" s="22"/>
+      <c r="G33" s="20"/>
+      <c r="H33" s="23"/>
+    </row>
+    <row r="34" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="17" t="n">
         <v>24</v>
       </c>
-      <c r="B33" s="21"/>
-      <c r="C33" s="22"/>
-      <c r="D33" s="23"/>
-      <c r="E33" s="22"/>
-      <c r="F33" s="23"/>
-      <c r="G33" s="24"/>
-    </row>
-    <row r="34" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="16" t="n">
+      <c r="B34" s="18"/>
+      <c r="C34" s="19" t="str">
+        <f aca="false">IF(B34="","",TEXT(B34,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="D34" s="24"/>
+      <c r="E34" s="25"/>
+      <c r="F34" s="26"/>
+      <c r="G34" s="24"/>
+      <c r="H34" s="27"/>
+    </row>
+    <row r="35" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="17" t="n">
         <v>25</v>
       </c>
-      <c r="B34" s="17"/>
-      <c r="C34" s="18"/>
-      <c r="D34" s="19"/>
-      <c r="E34" s="18"/>
-      <c r="F34" s="19"/>
-      <c r="G34" s="20"/>
-    </row>
-    <row r="35" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="16" t="n">
+      <c r="B35" s="18"/>
+      <c r="C35" s="19" t="str">
+        <f aca="false">IF(B35="","",TEXT(B35,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="D35" s="20"/>
+      <c r="E35" s="21"/>
+      <c r="F35" s="22"/>
+      <c r="G35" s="20"/>
+      <c r="H35" s="23"/>
+    </row>
+    <row r="36" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="17" t="n">
         <v>26</v>
       </c>
-      <c r="B35" s="21"/>
-      <c r="C35" s="22"/>
-      <c r="D35" s="23"/>
-      <c r="E35" s="22"/>
-      <c r="F35" s="23"/>
-      <c r="G35" s="24"/>
-    </row>
-    <row r="36" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="16" t="n">
+      <c r="B36" s="18"/>
+      <c r="C36" s="19" t="str">
+        <f aca="false">IF(B36="","",TEXT(B36,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="D36" s="24"/>
+      <c r="E36" s="25"/>
+      <c r="F36" s="26"/>
+      <c r="G36" s="24"/>
+      <c r="H36" s="27"/>
+    </row>
+    <row r="37" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="17" t="n">
         <v>27</v>
       </c>
-      <c r="B36" s="17"/>
-      <c r="C36" s="18"/>
-      <c r="D36" s="19"/>
-      <c r="E36" s="18"/>
-      <c r="F36" s="19"/>
-      <c r="G36" s="20"/>
-    </row>
-    <row r="37" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="16" t="n">
+      <c r="B37" s="18"/>
+      <c r="C37" s="19" t="str">
+        <f aca="false">IF(B37="","",TEXT(B37,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="D37" s="20"/>
+      <c r="E37" s="21"/>
+      <c r="F37" s="22"/>
+      <c r="G37" s="20"/>
+      <c r="H37" s="23"/>
+    </row>
+    <row r="38" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="17" t="n">
         <v>28</v>
       </c>
-      <c r="B37" s="21"/>
-      <c r="C37" s="22"/>
-      <c r="D37" s="23"/>
-      <c r="E37" s="22"/>
-      <c r="F37" s="23"/>
-      <c r="G37" s="24"/>
-    </row>
-    <row r="38" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="16" t="n">
+      <c r="B38" s="18"/>
+      <c r="C38" s="19" t="str">
+        <f aca="false">IF(B38="","",TEXT(B38,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="D38" s="24"/>
+      <c r="E38" s="25"/>
+      <c r="F38" s="26"/>
+      <c r="G38" s="24"/>
+      <c r="H38" s="27"/>
+    </row>
+    <row r="39" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="17" t="n">
         <v>29</v>
       </c>
-      <c r="B38" s="17"/>
-      <c r="C38" s="18"/>
-      <c r="D38" s="19"/>
-      <c r="E38" s="18"/>
-      <c r="F38" s="19"/>
-      <c r="G38" s="20"/>
-    </row>
-    <row r="39" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="16" t="n">
+      <c r="B39" s="18"/>
+      <c r="C39" s="19" t="str">
+        <f aca="false">IF(B39="","",TEXT(B39,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="D39" s="20"/>
+      <c r="E39" s="21"/>
+      <c r="F39" s="22"/>
+      <c r="G39" s="20"/>
+      <c r="H39" s="23"/>
+    </row>
+    <row r="40" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="17" t="n">
         <v>30</v>
       </c>
-      <c r="B39" s="21"/>
-      <c r="C39" s="22"/>
-      <c r="D39" s="23"/>
-      <c r="E39" s="22"/>
-      <c r="F39" s="23"/>
-      <c r="G39" s="24"/>
-    </row>
-    <row r="40" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="25" t="s">
-        <v>73</v>
-      </c>
-      <c r="B40" s="26"/>
-      <c r="C40" s="26"/>
-      <c r="D40" s="26"/>
-      <c r="E40" s="26"/>
+      <c r="B40" s="18"/>
+      <c r="C40" s="19" t="str">
+        <f aca="false">IF(B40="","",TEXT(B40,"ddd"))</f>
+        <v/>
+      </c>
+      <c r="D40" s="24"/>
+      <c r="E40" s="25"/>
       <c r="F40" s="26"/>
-      <c r="G40" s="27" t="n">
-        <f aca="false">SUM(G10:G39)</f>
+      <c r="G40" s="24"/>
+      <c r="H40" s="27"/>
+    </row>
+    <row r="41" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="28" t="s">
+        <v>74</v>
+      </c>
+      <c r="B41" s="29"/>
+      <c r="C41" s="29"/>
+      <c r="D41" s="29"/>
+      <c r="E41" s="29"/>
+      <c r="F41" s="29"/>
+      <c r="G41" s="29"/>
+      <c r="H41" s="30" t="n">
+        <f aca="false">SUM(H11:H40)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="42" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="28" t="s">
-        <v>74</v>
-      </c>
-      <c r="B42" s="28"/>
-      <c r="C42" s="28"/>
-      <c r="D42" s="28"/>
-      <c r="E42" s="28"/>
-      <c r="F42" s="28"/>
-      <c r="G42" s="28"/>
+    <row r="42" customFormat="false" ht="6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="43" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="31" t="s">
+        <v>75</v>
+      </c>
+      <c r="B43" s="31"/>
+      <c r="C43" s="31"/>
+      <c r="D43" s="31"/>
+      <c r="E43" s="31"/>
+      <c r="F43" s="31"/>
+      <c r="G43" s="31"/>
+      <c r="H43" s="31"/>
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A2:H2"/>
     <mergeCell ref="B5:D5"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="A7:G7"/>
-    <mergeCell ref="A42:G42"/>
+    <mergeCell ref="F6:H6"/>
+    <mergeCell ref="A8:H8"/>
+    <mergeCell ref="A43:H43"/>
   </mergeCells>
   <dataValidations count="4">
-    <dataValidation allowBlank="true" error="Choose from: Design, Drafting, Coordination, Meetings, Admin, Site, Other" errorStyle="stop" errorTitle="Invalid Category" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="E10:E39" type="list">
-      <formula1>"Design,Drafting,Coordination,Meetings,Admin,Site,Other"</formula1>
+    <dataValidation allowBlank="true" error="Please select from the dropdown list." errorStyle="stop" errorTitle="Invalid Category" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="F11:F40" type="list">
+      <formula1>_Lists!$A$1:$A$11</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" error="Choose from: Mon, Tue, Wed, Thu, Fri, Sat, Sun" errorStyle="stop" errorTitle="Invalid Day" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="C10:C39" type="list">
-      <formula1>"Mon,Tue,Wed,Thu,Fri,Sat,Sun"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" error="Hours must be a decimal number between 0 and 24 (e.g. 7.5)" errorStyle="stop" errorTitle="Invalid Hours" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="G10:G39" type="decimal">
+    <dataValidation allowBlank="true" error="Enter a decimal number between 0 and 24 (e.g. 7.5)" errorStyle="stop" errorTitle="Invalid Hours" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H11:H40" type="decimal">
       <formula1>0</formula1>
       <formula2>24</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" error="Please enter a valid date." errorStyle="stop" errorTitle="Invalid Date" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B10:B39" type="date">
+    <dataValidation allowBlank="true" error="Please enter a valid date." errorStyle="stop" errorTitle="Invalid Date" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B11:B40" type="date">
+      <formula1>0</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" error="Enter the Monday date for the week." errorStyle="stop" errorTitle="Invalid Date" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B6" type="date">
       <formula1>0</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -1764,4 +1937,78 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:A11"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="0" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="0" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="0" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="0" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="0" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="0" t="s">
+        <v>51</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>